<commit_message>
Atualizações de resultados na VIT 15/05
</commit_message>
<xml_diff>
--- a/Project_CNN/ResNet/Results/Unified Training Metrics - ResNet BS32 500EPS.xlsx
+++ b/Project_CNN/ResNet/Results/Unified Training Metrics - ResNet BS32 500EPS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci_wawp\Desktop\Arquivos\Mestrado\Projeto-Classificadores\Project_CNN\ResNet\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5618B1B-F012-4D39-A8E0-4CF949A1CC2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A0CCC5B-8EED-4B30-ABC9-44D754A8E328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -222,7 +222,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="pt-BR" baseline="0"/>
-              <a:t>Accuracy Curves</a:t>
+              <a:t>Curvas de Acurácia no treino</a:t>
             </a:r>
             <a:endParaRPr lang="pt-BR"/>
           </a:p>
@@ -2024,14 +2024,16 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="pt-BR"/>
-                  <a:t>Accuracy</a:t>
+                  <a:rPr lang="pt-BR" sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Acurácia (%)</a:t>
                 </a:r>
-                <a:r>
-                  <a:rPr lang="pt-BR" baseline="0"/>
-                  <a:t> (%)</a:t>
-                </a:r>
-                <a:endParaRPr lang="pt-BR"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -2218,14 +2220,16 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="pt-BR"/>
-              <a:t>Validation</a:t>
+              <a:rPr lang="pt-BR" sz="2400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Curvas de Acurácia na validação</a:t>
             </a:r>
-            <a:r>
-              <a:rPr lang="pt-BR" baseline="0"/>
-              <a:t> Accuracy Curves</a:t>
-            </a:r>
-            <a:endParaRPr lang="pt-BR"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -4035,7 +4039,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="pt-BR"/>
-                  <a:t>Accuracy</a:t>
+                  <a:t>Acurácia</a:t>
                 </a:r>
                 <a:r>
                   <a:rPr lang="pt-BR" baseline="0"/>
@@ -4229,7 +4233,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="pt-BR"/>
-              <a:t>Loss Curves</a:t>
+              <a:t>Curvas de Perda no treino</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -5908,7 +5912,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="pt-BR"/>
-                  <a:t>Epochs</a:t>
+                  <a:t>Épocas</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -6026,7 +6030,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="pt-BR"/>
-                  <a:t>Loss</a:t>
+                  <a:t>Perda</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -6212,12 +6216,15 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="pt-BR"/>
-              <a:t>Validation</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="pt-BR" baseline="0"/>
-              <a:t> Loss Curves</a:t>
+              <a:rPr lang="pt-BR" sz="2400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Curvas de Perda na validação</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -7895,9 +7902,17 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="pt-BR"/>
-                  <a:t>Epochs</a:t>
+                  <a:rPr lang="pt-BR" sz="2400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Épocas</a:t>
                 </a:r>
+                <a:endParaRPr lang="pt-BR"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -8013,8 +8028,15 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="pt-BR"/>
-                  <a:t>Loss</a:t>
+                  <a:rPr lang="pt-BR" sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Perda</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -10395,15 +10417,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>24</xdr:col>
-      <xdr:colOff>792062</xdr:colOff>
-      <xdr:row>59</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>2847</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>492473</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>159991</xdr:rowOff>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>458968</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>164937</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -10430,16 +10452,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>490931</xdr:colOff>
-      <xdr:row>59</xdr:row>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>463716</xdr:colOff>
+      <xdr:row>58</xdr:row>
       <xdr:rowOff>1421</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>34</xdr:col>
-      <xdr:colOff>27214</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>161412</xdr:rowOff>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>824105</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>166357</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -10469,15 +10491,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>24</xdr:col>
-      <xdr:colOff>791440</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>165086</xdr:rowOff>
+      <xdr:colOff>2226</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>165087</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>490931</xdr:colOff>
-      <xdr:row>112</xdr:row>
-      <xdr:rowOff>133349</xdr:rowOff>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>457088</xdr:colOff>
+      <xdr:row>101</xdr:row>
+      <xdr:rowOff>138523</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -10504,16 +10526,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>490931</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>463716</xdr:colOff>
+      <xdr:row>79</xdr:row>
       <xdr:rowOff>162636</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>34</xdr:col>
-      <xdr:colOff>26294</xdr:colOff>
-      <xdr:row>112</xdr:row>
-      <xdr:rowOff>130899</xdr:rowOff>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>830035</xdr:colOff>
+      <xdr:row>101</xdr:row>
+      <xdr:rowOff>136072</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>